<commit_message>
Fix FINAL_EXP.xlsx formatting: borders and green fill on new rows
Match existing row styling (thin borders, green metric columns E-J).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FINAL_EXP.xlsx
+++ b/FINAL_EXP.xlsx
@@ -32,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,10 @@
       <family val="2"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -92,7 +96,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -115,11 +119,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -137,6 +147,8 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1597,376 +1609,376 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>weight_sparsity_5500</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>RigL-style weight sparsity (30%) with gradient-guided regrowth</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Dynamic sparse training recycles dead weights; may improve generalization at 0.72B scale</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="10" t="n">
         <v>3.5097</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="10" t="n">
         <v>33.43823480863127</v>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>78,325,183</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>17.76%</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>22.0%</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="9" t="inlineStr">
         <is>
           <t>checkpoints/weight_sparsity_5500.pt</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr"/>
+      <c r="M17" s="9" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/1hyu3bd6</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="N17" s="9" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>data_optimization_5500_rerun</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>QA data augmentation (4,681 QA samples mixed at 10% ratio)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>QA-format data improves comprehension; corrected to 0.72B (original was 0.09B on 1 GPU)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="10" t="n">
         <v>3.4568</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="10" t="n">
         <v>31.71532491911631</v>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>51.0%</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K18" s="9" t="inlineStr">
         <is>
           <t>checkpoints/data_optimization_5500_rerun.pt</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr"/>
+      <c r="M18" s="9" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/ader9y8r</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N18" s="9" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>everything_optimized_5500_rerun</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>All tricks: Muon + ReLU2 FFN + QK norm + softcap + resid scalars + QA data</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>All modifications at 0.72B; corrected from 0.09B (original was 1 GPU)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="10" t="n">
         <v>3.2661</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="10" t="n">
         <v>26.20892495768922</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>95,246,608</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="10" t="inlineStr">
         <is>
           <t>72.0%</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K19" s="9" t="inlineStr">
         <is>
           <t>checkpoints/everything_optimized_5500_rerun.pt</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr"/>
+      <c r="M19" s="9" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/friejl4l</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="N19" s="9" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>everything_50M_rerun</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>All tricks combined (50M tokens) — reproducibility rerun</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Rerun to verify: original=65%, Asher=25%. Rerun=69% — confirms original results</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="10" t="n">
         <v>3.8948</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="10" t="n">
         <v>49.14622313506688</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>95,246,608</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="10" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="10" t="inlineStr">
         <is>
           <t>69.0%</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K20" s="9" t="inlineStr">
         <is>
           <t>checkpoints/everything_50M_rerun.pt</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr">
+      <c r="L20" s="9" t="inlineStr"/>
+      <c r="M20" s="9" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/jf0s3p1l</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="N20" s="9" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>copy_gate_5500_rerun</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Copy gate (769 params) on frozen baseline_10x_less, retrained on correct checkpoint</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Copy mechanism for direct token recall; p_copy converged to 4.1%</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="10" t="n">
         <v>3.4151</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="10" t="n">
         <v>30.41999127459776</v>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>95,247,361</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="10" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>28.0%</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K21" s="9" t="inlineStr">
         <is>
           <t>checkpoints/copy_gate_5500.pt</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
+      <c r="L21" s="9" t="inlineStr"/>
+      <c r="M21" s="9" t="inlineStr"/>
+      <c r="N21" s="9" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>copy_gate_50M</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Copy gate (769 params) on frozen baseline_50M_retrain</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>Copy mechanism at smallest scale; p_copy converged to 5.4%</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="10" t="n">
         <v>4.2903</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="10" t="n">
         <v>72.98836172400216</v>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="10" t="inlineStr">
         <is>
           <t>114,121,729</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="10" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="10" t="inlineStr">
         <is>
           <t>1.0%</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="K22" s="9" t="inlineStr">
         <is>
           <t>checkpoints/copy_gate_50M.pt</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
+      <c r="L22" s="9" t="inlineStr"/>
+      <c r="M22" s="9" t="inlineStr"/>
+      <c r="N22" s="9" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>

</xml_diff>

<commit_message>
Update FINAL_EXP.xlsx with true-everything results and striped row colors
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FINAL_EXP.xlsx
+++ b/FINAL_EXP.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dataset_Overview" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Examples_baseline" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Examples_baseline_10x_less" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Examples_relu2_ffn_5500" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Examples_muon_optimizer_5500" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Examples_attn_residual_tricks_5" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Examples_copy_gate" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Examples_everything_optimized_5" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Examples_data_optimization_5500" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Examples_relu2_50M" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Examples_everything_50M" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Examples_baseline_50M" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Examples_data_opt_50M" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Examples_muon_50M" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Examples_attn_tricks_50M" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Examples_weight_sparsity_50M" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Experiments" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset_Overview" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_baseline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_baseline_10x_less" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_relu2_ffn_5500" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_muon_optimizer_5500" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_attn_residual_tricks_5" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_copy_gate" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_everything_optimized_5" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_data_optimization_5500" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_relu2_50M" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_everything_50M" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_baseline_50M" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_data_opt_50M" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_muon_50M" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_attn_tricks_50M" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples_weight_sparsity_50M" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -70,7 +70,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +93,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8E8E8"/>
+        <bgColor rgb="FFE8E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD5DDD0"/>
+        <bgColor rgb="FFD5DDD0"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -149,6 +161,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="8" min="1" max="1"/>
@@ -601,1200 +629,1200 @@
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" s="8">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>None (baseline SimpleTransformer)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Establish baseline performance</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="12" t="n">
         <v>3.0463</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="12" t="n">
         <v>21.0373620046153</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>7.21B</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>40.0%</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>checkpoints/baseline_full_8gpu.pt</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>https://85e7746ab5c7cab600.gradio.live</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/dzpejlpz</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" s="11" t="inlineStr">
         <is>
           <t>2026-02-21 23:39</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" s="8">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>baseline_10x_less</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Same architecture, 10x less data (5,500 steps instead of 55,000)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Measure impact of data scaling on Story QA accuracy</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" s="14" t="n">
         <v>3.4181</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="14" t="n">
         <v>30.51138827537498</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="14" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="14" t="inlineStr">
         <is>
           <t>18.0%</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="13" t="inlineStr">
         <is>
           <t>checkpoints/baseline_10x_less.pt</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="L3" s="13" t="n"/>
+      <c r="M3" s="13" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/gyr7s6bh</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N3" s="13" t="inlineStr">
         <is>
           <t>2026-02-21 23:41</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1" s="8">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>relu2_ffn_5500</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>ReLU² FFN (2 matrices, d_ff=3072) replacing SwiGLU FFN (3 matrices, d_ff=2048)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>ReLU² uses 2 matrices instead of 3, larger d_ff for same param budget; squared ReLU encourages activation sparsity</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="14" t="n">
         <v>3.387</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="14" t="n">
         <v>29.57708777694624</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="14" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="14" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="14" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="14" t="inlineStr">
         <is>
           <t>32.0%</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>checkpoints/relu2_ffn_5500.pt</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="13" t="inlineStr">
         <is>
           <t>https://5f7c79094dcad8ba5b.gradio.live</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" s="13" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/568s23ch</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N4" s="13" t="inlineStr">
         <is>
           <t>2026-02-22 01:27</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1" s="8">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>muon_optimizer_5500</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Muon optimizer (MuonAdamW) replacing AdamW, with warmup/constant/warmdown LR schedule</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>Muon converges faster for matrix params via orthogonal updates; warmup→constant→warmdown schedule is gentler than linear decay</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="14" t="n">
         <v>3.2403</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="14" t="n">
         <v>25.54138301300812</v>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="14" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="14" t="inlineStr">
         <is>
           <t>34.0%</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="13" t="inlineStr">
         <is>
           <t>checkpoints/muon_optimizer_5500.pt</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>https://f3f8d2eba642a2615f.gradio.live</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M5" s="13" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/ejft5bl0</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N5" s="13" t="inlineStr">
         <is>
           <t>2026-02-22 01:28</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" s="8">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>attn_residual_tricks_5500</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>QK normalization + logit softcapping (15.0) + per-layer residual scalars</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>QK norm stabilizes attention; softcap prevents logit explosion; residual scalars improve gradient flow</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="12" t="n">
         <v>3.399</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="12" t="n">
         <v>29.93415092440687</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>95,246,608</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="12" t="inlineStr">
         <is>
           <t>0.63B</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>30.0%</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>checkpoints/attn_residual_tricks_5500.pt</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L6" s="11" t="inlineStr">
         <is>
           <t>https://fe6d3bfe2620e6d445.gradio.live</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M6" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/q0l3uvz3</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 01:29</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" s="8">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>copy_gate</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Copy gate mechanism (769 trainable params on frozen baseline)</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Learnable gate blending generation and copy distributions; helps with factual recall by copying from context</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="12" t="n">
         <v>3.0444</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="12" t="n">
         <v>20.99742896520715</v>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>0.63B</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>34.0%</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>checkpoints/copy_gate.pt</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="11" t="inlineStr">
         <is>
           <t>https://7a77077e94af69a677.gradio.live</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="M7" s="11" t="n"/>
+      <c r="N7" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 01:40</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" s="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>everything_optimized_5500</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>All modifications: Muon optimizer + ReLU2 FFN + QK norm + softcap + residual scalars + QA data</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>Combining all individually-tested tricks should yield best val_loss</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="12" t="n">
         <v>3.7473</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="12" t="n">
         <v>42.4064299286102</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>95,246,608</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>0.63B</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>63.0%</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>checkpoints/everything_optimized_5500.pt</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L8" s="11" t="inlineStr">
         <is>
           <t>https://931517c021bb1e6624.gradio.live</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M8" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/hu9igyf8</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N8" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 02:48</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" s="8">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>data_optimization_5500</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>QA data augmentation (4299 QA samples mixed at 10% ratio)</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Augmenting FineWeb-edu with Story QA-style data should improve factual recall and QA accuracy</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="14" t="n">
         <v>4.0886</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="14" t="n">
         <v>59.65631437354176</v>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>0.09B</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="14" t="inlineStr">
         <is>
           <t>15.0%</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K9" s="13" t="inlineStr">
         <is>
           <t>checkpoints/data_optimization_5500.pt</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L9" s="13" t="inlineStr">
         <is>
           <t>https://0995494f3fbd83dae9.gradio.live</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M9" s="13" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/4o92o59s</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N9" s="13" t="inlineStr">
         <is>
           <t>2026-02-22 05:24</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" s="8">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>relu2_50M</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>ReLU2 FFN only (50M tokens)</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Test ReLU2 FFN in isolation at 50M tokens</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="12" t="n">
         <v>4.3105</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="12" t="n">
         <v>74.47771849142779</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="12" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>3.0%</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>checkpoints/relu2_50M.pt</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L10" s="11" t="inlineStr">
         <is>
           <t>https://56622a26ee166f1dcd.gradio.live</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M10" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/n84fk7gy</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N10" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 05:55</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" s="8">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>everything_50M</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>All modifications combined (50M tokens)</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Test all tricks combined at 50M tokens</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="12" t="n">
         <v>3.8891</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="12" t="n">
         <v>48.86688652882823</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>65.0%</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>checkpoints/everything_50M.pt</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L11" s="11" t="inlineStr">
         <is>
           <t>https://d902716b9dc0f3268e.gradio.live</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M11" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/8gi63uty</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N11" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 05:56</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" s="8">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>baseline_50M</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>None (baseline, 50M tokens, d_ff=3072)</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>Baseline reference at 50M token budget</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="12" t="n">
         <v>4.3632</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="12" t="n">
         <v>78.50795835749679</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>checkpoints/baseline_50M.pt</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>https://539ed58d679565a51e.gradio.live</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M12" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/ppmqwsr9</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N12" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 06:06</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" s="8">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>data_opt_50M</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>QA data augmentation only (50M tokens, d_ff=3072)</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Test QA data mixing in isolation at 50M tokens</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="12" t="n">
         <v>4.3795</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="12" t="n">
         <v>79.79812436647308</v>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="12" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J13" s="12" t="inlineStr">
         <is>
           <t>1.0%</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>checkpoints/data_opt_50M.pt</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="11" t="inlineStr">
         <is>
           <t>https://8ed4339d026385f523.gradio.live</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M13" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/o81o5dxt</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N13" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 06:06</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" s="8">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>muon_50M</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Muon optimizer only (50M tokens, d_ff=3072)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>Test Muon optimizer in isolation at 50M tokens</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="12" t="n">
         <v>3.9545</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="12" t="n">
         <v>52.16960262083392</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" s="12" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J14" s="12" t="inlineStr">
         <is>
           <t>8.0%</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>checkpoints/muon_50M.pt</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>https://9706ee357bb10edbb1.gradio.live</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M14" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/kg37qul9</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N14" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 06:06</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1" s="8">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>attn_tricks_50M</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>QK norm + softcap + resid scalars only (50M tokens, d_ff=3072)</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Test attention/residual tricks in isolation at 50M tokens</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="12" t="n">
         <v>4.2931</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="12" t="n">
         <v>73.19301551843442</v>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>463</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J15" s="12" t="inlineStr">
         <is>
           <t>1.0%</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>checkpoints/attn_tricks_50M.pt</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L15" s="11" t="inlineStr">
         <is>
           <t>https://28d0b8191490642ff9.gradio.live</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M15" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/jqzpd7zv</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N15" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 06:06</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" s="8">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>weight_sparsity_50M</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Weight sparsity 30% (RigL-style prune-regrow)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>Dynamic sparse training recycles dead weights to where gradients are largest, maintaining quality with fewer effective params</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="12" t="n">
         <v>4.5154</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="12" t="n">
         <v>91.41412435997725</v>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>79,031,706</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>17.02%</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="12" t="inlineStr">
         <is>
           <t>0.05B</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J16" s="12" t="inlineStr">
         <is>
           <t>2.0%</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>checkpoints/weight_sparsity_50M.pt</t>
         </is>
       </c>
-      <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="L16" s="11" t="n"/>
+      <c r="M16" s="11" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/iaoigghe</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N16" s="11" t="inlineStr">
         <is>
           <t>2026-02-22 06:10</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>weight_sparsity_5500</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>RigL-style weight sparsity (30%) with gradient-guided regrowth</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>Dynamic sparse training recycles dead weights; may improve generalization at 0.72B scale</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="16" t="n">
         <v>3.5097</v>
       </c>
-      <c r="F17" s="10" t="n">
+      <c r="F17" s="16" t="n">
         <v>33.43823480863127</v>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>78,325,183</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>17.76%</t>
         </is>
       </c>
-      <c r="I17" s="10" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="J17" s="16" t="inlineStr">
         <is>
           <t>22.0%</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr">
+      <c r="K17" s="15" t="inlineStr">
         <is>
           <t>checkpoints/weight_sparsity_5500.pt</t>
         </is>
       </c>
-      <c r="L17" s="9" t="inlineStr"/>
-      <c r="M17" s="9" t="inlineStr">
+      <c r="L17" s="15" t="inlineStr"/>
+      <c r="M17" s="15" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/1hyu3bd6</t>
         </is>
       </c>
-      <c r="N17" s="9" t="inlineStr">
+      <c r="N17" s="15" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>data_optimization_5500_rerun</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>QA data augmentation (4,681 QA samples mixed at 10% ratio)</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <t>QA-format data improves comprehension; corrected to 0.72B (original was 0.09B on 1 GPU)</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="16" t="n">
         <v>3.4568</v>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="F18" s="16" t="n">
         <v>31.71532491911631</v>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>95,246,592</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I18" s="10" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J18" s="10" t="inlineStr">
+      <c r="J18" s="16" t="inlineStr">
         <is>
           <t>51.0%</t>
         </is>
       </c>
-      <c r="K18" s="9" t="inlineStr">
+      <c r="K18" s="15" t="inlineStr">
         <is>
           <t>checkpoints/data_optimization_5500_rerun.pt</t>
         </is>
       </c>
-      <c r="L18" s="9" t="inlineStr"/>
-      <c r="M18" s="9" t="inlineStr">
+      <c r="L18" s="15" t="inlineStr"/>
+      <c r="M18" s="15" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/ader9y8r</t>
         </is>
       </c>
-      <c r="N18" s="9" t="inlineStr">
+      <c r="N18" s="15" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>everything_optimized_5500_rerun</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>All tricks: Muon + ReLU2 FFN + QK norm + softcap + resid scalars + QA data</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>All modifications at 0.72B; corrected from 0.09B (original was 1 GPU)</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>COMPLETE ✓ GOAL</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="16" t="n">
         <v>3.2661</v>
       </c>
-      <c r="F19" s="10" t="n">
+      <c r="F19" s="16" t="n">
         <v>26.20892495768922</v>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>95,246,608</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I19" s="10" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J19" s="10" t="inlineStr">
+      <c r="J19" s="16" t="inlineStr">
         <is>
           <t>72.0%</t>
         </is>
       </c>
-      <c r="K19" s="9" t="inlineStr">
+      <c r="K19" s="15" t="inlineStr">
         <is>
           <t>checkpoints/everything_optimized_5500_rerun.pt</t>
         </is>
       </c>
-      <c r="L19" s="9" t="inlineStr"/>
-      <c r="M19" s="9" t="inlineStr">
+      <c r="L19" s="15" t="inlineStr"/>
+      <c r="M19" s="15" t="inlineStr">
         <is>
           <t>https://wandb.ai/jinyoungkim927/weightless/runs/friejl4l</t>
         </is>
       </c>
-      <c r="N19" s="9" t="inlineStr">
+      <c r="N19" s="15" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
@@ -1865,60 +1893,60 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>copy_gate_5500_rerun</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Copy gate (769 params) on frozen baseline_10x_less, retrained on correct checkpoint</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>Copy mechanism for direct token recall; p_copy converged to 4.1%</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="16" t="n">
         <v>3.4151</v>
       </c>
-      <c r="F21" s="10" t="n">
+      <c r="F21" s="16" t="n">
         <v>30.41999127459776</v>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>95,247,361</t>
         </is>
       </c>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>0.00%</t>
         </is>
       </c>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>0.72B</t>
         </is>
       </c>
-      <c r="J21" s="10" t="inlineStr">
+      <c r="J21" s="16" t="inlineStr">
         <is>
           <t>28.0%</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="K21" s="15" t="inlineStr">
         <is>
           <t>checkpoints/copy_gate_5500.pt</t>
         </is>
       </c>
-      <c r="L21" s="9" t="inlineStr"/>
-      <c r="M21" s="9" t="inlineStr"/>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="L21" s="15" t="inlineStr"/>
+      <c r="M21" s="15" t="inlineStr"/>
+      <c r="N21" s="15" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
         </is>
@@ -1981,6 +2009,134 @@
       <c r="N22" s="9" t="inlineStr">
         <is>
           <t>2026-02-27 05:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>true_everything_50M</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>True everything (all mods + QA data + sparsity + copy gate)</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Does combining ALL modifications (incl. sparsity + copy gate) improve Story QA beyond everything_optimized?</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>3.9465</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>51.75391078423441</v>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>78,913,436</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>17.15%</t>
+        </is>
+      </c>
+      <c r="I23" s="18" t="inlineStr">
+        <is>
+          <t>0.05B</t>
+        </is>
+      </c>
+      <c r="J23" s="18" t="inlineStr">
+        <is>
+          <t>57.0%</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="inlineStr">
+        <is>
+          <t>checkpoints/true_everything_copy_gate_50M.pt</t>
+        </is>
+      </c>
+      <c r="L23" s="17" t="n"/>
+      <c r="M23" s="17" t="inlineStr">
+        <is>
+          <t>https://wandb.ai/jinyoungkim927/weightless/runs/t50rm09f</t>
+        </is>
+      </c>
+      <c r="N23" s="17" t="inlineStr">
+        <is>
+          <t>2026-02-27 06:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>true_everything_no_qa_50M</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>True everything (all mods + sparsity + copy gate, NO QA data)</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Isolate architectural mods from QA data: do sparsity + copy gate help without QA augmentation?</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="n">
+        <v>3.9429</v>
+      </c>
+      <c r="F24" s="18" t="n">
+        <v>51.56793166867657</v>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>78,896,305</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>17.17%</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>0.05B</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>15.0%</t>
+        </is>
+      </c>
+      <c r="K24" s="17" t="inlineStr">
+        <is>
+          <t>checkpoints/true_everything_no_qa_copy_gate_50M.pt</t>
+        </is>
+      </c>
+      <c r="L24" s="17" t="n"/>
+      <c r="M24" s="17" t="inlineStr">
+        <is>
+          <t>https://wandb.ai/jinyoungkim927/weightless/runs/kr80al8r</t>
+        </is>
+      </c>
+      <c r="N24" s="17" t="inlineStr">
+        <is>
+          <t>2026-02-27 06:24</t>
         </is>
       </c>
     </row>

</xml_diff>